<commit_message>
Remove second, incomplete stale-vocabulary fragment in Read Me sheet
Found while verifying DT's claim that this workbook uses the locked
family vocabulary throughout (briefs/2026-07-26-prioritization-v1-resolution/):
Read Me!A25:C31 carried a second, abandoned A-E orientation lookup
using the old Initial/Emerging/... terms, missed in the earlier
Reference-sheet fix. Incomplete on its own terms (no D row, no C/E
orientation words) and fully redundant with the now-corrected
Reference sheet table -- removed rather than repaired into a duplicate.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AI_Native_Product_Prioritization_Maturity_Model_v1.0.xlsx
+++ b/AI_Native_Product_Prioritization_Maturity_Model_v1.0.xlsx
@@ -745,7 +745,7 @@
               <a:defRPr sz="675"/>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -1652,11 +1652,7 @@
       <c r="Z24" s="1" t="n"/>
     </row>
     <row r="25" ht="43.5" customHeight="1">
-      <c r="A25" s="43" t="inlineStr">
-        <is>
-          <t>A–E orientation</t>
-        </is>
-      </c>
+      <c r="A25" s="43" t="n"/>
       <c r="B25" s="43" t="n"/>
       <c r="I25" s="1" t="n"/>
       <c r="J25" s="1" t="n"/>
@@ -1678,16 +1674,8 @@
       <c r="Z25" s="1" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="47" t="inlineStr">
-        <is>
-          <t>Grade</t>
-        </is>
-      </c>
-      <c r="B26" s="47" t="inlineStr">
-        <is>
-          <t>Orientation</t>
-        </is>
-      </c>
+      <c r="A26" s="47" t="n"/>
+      <c r="B26" s="47" t="n"/>
       <c r="I26" s="1" t="n"/>
       <c r="J26" s="1" t="n"/>
       <c r="K26" s="1" t="n"/>
@@ -1708,16 +1696,8 @@
       <c r="Z26" s="1" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="28" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="B27" s="48" t="inlineStr">
-        <is>
-          <t>Initial</t>
-        </is>
-      </c>
+      <c r="A27" s="28" t="n"/>
+      <c r="B27" s="48" t="n"/>
       <c r="I27" s="1" t="n"/>
       <c r="J27" s="1" t="n"/>
       <c r="K27" s="1" t="n"/>
@@ -1738,21 +1718,9 @@
       <c r="Z27" s="1" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="45" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="B28" s="45" t="inlineStr">
-        <is>
-          <t>Emerging</t>
-        </is>
-      </c>
-      <c r="C28" s="45" t="inlineStr">
-        <is>
-          <t>Repeatable method with selective AI assistance and uneven governance.</t>
-        </is>
-      </c>
+      <c r="A28" s="45" t="n"/>
+      <c r="B28" s="45" t="n"/>
+      <c r="C28" s="45" t="n"/>
       <c r="I28" s="1" t="n"/>
       <c r="J28" s="1" t="n"/>
       <c r="K28" s="1" t="n"/>
@@ -1773,11 +1741,7 @@
       <c r="Z28" s="1" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="49" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
+      <c r="A29" s="49" t="n"/>
       <c r="I29" s="1" t="n"/>
       <c r="J29" s="1" t="n"/>
       <c r="K29" s="1" t="n"/>
@@ -1818,11 +1782,7 @@
       <c r="Z30" s="1" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="46" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
+      <c r="A31" s="46" t="n"/>
       <c r="I31" s="1" t="n"/>
       <c r="J31" s="1" t="n"/>
       <c r="K31" s="1" t="n"/>

</xml_diff>